<commit_message>
feat(painel): relatorios ABNT por evento+geral, carga horaria e palestrante em modal
- Exportacoes CSV/PDF/Excel/PPTX em padrao ABNT (capa, sumario, introducao, numeracao, figuras com fonte e data de extracao); conteudo por evento e consolidado conforme filtro de evento/secretaria; sem listas nominais; sem travessao.
- Auditoria: vinculo (efetivo/comissionado) por servidor unico com bucket 'Nao informado'; 'Ocupacao' do funil renomeada para preenchimento de vagas.
- Informacao de Cargos removida das paginas e dos arquivos (mantida dormente).
- Carga horaria por evento (eventos-meta.json) propagada ao build, ao detalhe do evento, ao perfil do servidor e ao certificado; data do Ciclo corrigida (17/05).
- Palestrantes: navegacao so com Galeria; Novo/editar abrem modal com etapas.
- Secretarias: grafico e ranking de faltas por secretaria.
</commit_message>
<xml_diff>
--- a/assets/docs/relatorios/ciclo-de-debates-pl-por-elas-2026-05/turma 1/participantes.xlsx
+++ b/assets/docs/relatorios/ciclo-de-debates-pl-por-elas-2026-05/turma 1/participantes.xlsx
@@ -6,7 +6,7 @@
     <sheet name="Lista de participantes" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Lista de participantes'!A1:I37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Lista de participantes'!A1:I40</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -35,12 +35,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="5">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -404,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I40"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -437,16 +433,16 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Ana Paula Silva Diniz</v>
+        <v>Alexsandra Torres Vitorino</v>
       </c>
       <c r="B2" t="str">
-        <v>apsd40063@gmail.com</v>
+        <v>leleka.vitorino@gmail.com</v>
       </c>
       <c r="C2" t="str">
-        <v>Secretaria Municipal de Bem Estar</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D2" t="str">
-        <v>DCA 1</v>
+        <v>Coordenação</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -455,10 +451,10 @@
         <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G2" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-04-07 17:56:42</v>
+        <v>2026-04-07 18:07:15</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -466,16 +462,16 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Elisângel Mesquita de Oliveira</v>
+        <v>Sonila Marques</v>
       </c>
       <c r="B3" t="str">
-        <v>elisangela31mesquita@gmail.com</v>
+        <v>sonila.marques@gmail.com</v>
       </c>
       <c r="C3" t="str">
-        <v>Controladoria Geral do Município</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D3" t="str">
-        <v>Gerente Controle Interno</v>
+        <v>Farmacêutica</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -484,10 +480,10 @@
         <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G3" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-04-07 18:01:44</v>
+        <v>2026-04-09 17:04:07</v>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -495,28 +491,28 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Daniela Mara de Oliveira Roberto Roberto</v>
+        <v>Maria Inês Clemente Bassouto Estevam</v>
       </c>
       <c r="B4" t="str">
-        <v>danipl22@yahoo.com.br</v>
+        <v>maria.estevam@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C4" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D4" t="str">
-        <v>Técnico de Enfermagem</v>
+        <v>Gerente de Saúde Ocupacional</v>
       </c>
       <c r="E4" t="str">
         <v/>
       </c>
       <c r="F4" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G4" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-04-07 18:02:05</v>
+        <v>2026-04-10 11:04:12</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -524,16 +520,16 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Alexsandra Torres Vitorino</v>
+        <v>Polyana Parreiras</v>
       </c>
       <c r="B5" t="str">
-        <v>leleka.vitorino@gmail.com</v>
+        <v>PSPARREIRAS@GMAIL.COM</v>
       </c>
       <c r="C5" t="str">
         <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D5" t="str">
-        <v>Coordenação</v>
+        <v>Supervisora</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -542,10 +538,10 @@
         <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G5" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-04-07 18:07:15</v>
+        <v>2026-04-10 11:04:23</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -553,16 +549,16 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Priscilla Gomes Rodrigues</v>
+        <v>Priscila Malaquias</v>
       </c>
       <c r="B6" t="str">
-        <v>priscillagomesr@gmail.com</v>
+        <v>priscila.malaquiass@gmail.com</v>
       </c>
       <c r="C6" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Governo</v>
       </c>
       <c r="D6" t="str">
-        <v>Coordenação</v>
+        <v>Analista  Administrativo</v>
       </c>
       <c r="E6" t="str">
         <v/>
@@ -571,10 +567,10 @@
         <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G6" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-04-07 18:09:20</v>
+        <v>2026-04-10 11:05:06</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -582,16 +578,16 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Dirciana Fátima Silva</v>
+        <v>Adriana Cristiene Demétrio</v>
       </c>
       <c r="B7" t="str">
-        <v>dircianafatimademourasilva@gmail.com</v>
+        <v>adriana.demetrio@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C7" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D7" t="str">
-        <v>Auxiliar Administrativo</v>
+        <v>Assistente Administrativo</v>
       </c>
       <c r="E7" t="str">
         <v/>
@@ -600,10 +596,10 @@
         <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G7" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-04-07 18:13:19</v>
+        <v>2026-04-10 11:12:05</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -611,16 +607,16 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Maria de Fátima Gonçalves Cardoso</v>
+        <v>Tássia Junqueira</v>
       </c>
       <c r="B8" t="str">
-        <v>mfgcardoso445@gmail.com</v>
+        <v>tassia.junqueira@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C8" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D8" t="str">
-        <v>Agente de saude</v>
+        <v>GERENTE</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -629,10 +625,10 @@
         <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G8" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-04-07 18:14:10</v>
+        <v>2026-04-10 14:53:23</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -640,28 +636,28 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Lais Macedo Bonfim Rocha</v>
+        <v>Ana Beatriz Souza de Jesus</v>
       </c>
       <c r="B9" t="str">
-        <v>lmbrocha@pedroleopoldo.mg.gov.br</v>
+        <v>ana.jesus@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C9" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D9" t="str">
-        <v>Técnica em Radiologia/Supervisora das Técnicas Radiológicas</v>
+        <v>Analista Administrativo</v>
       </c>
       <c r="E9" t="str">
         <v/>
       </c>
       <c r="F9" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G9" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H9" t="str">
-        <v>2026-04-07 18:40:08</v>
+        <v>2026-04-10 15:08:22</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -669,16 +665,16 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Jeane Fraga dos Santos Pereira</v>
+        <v>Renata dos Santos Nestor</v>
       </c>
       <c r="B10" t="str">
-        <v>pereira_jeane2016@yahoo.com.br</v>
+        <v>renata.nestor@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C10" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D10" t="str">
-        <v>Técnica de Enfermagem</v>
+        <v>DCA 1</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -687,10 +683,10 @@
         <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G10" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H10" t="str">
-        <v>2026-04-07 18:41:50</v>
+        <v>2026-04-10 15:12:25</v>
       </c>
       <c r="I10" t="str">
         <v/>
@@ -698,28 +694,28 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Libânia Cássia Alves Alves</v>
+        <v>Olga Arruda</v>
       </c>
       <c r="B11" t="str">
-        <v>libaniacassia@hotmail.com</v>
+        <v>olga_arruda@hotmail.com</v>
       </c>
       <c r="C11" t="str">
-        <v>Secretaria Municipal de Governo</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D11" t="str">
-        <v>Coordenadora de projeto</v>
+        <v>Supervisora</v>
       </c>
       <c r="E11" t="str">
         <v/>
       </c>
       <c r="F11" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G11" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-04-07 18:43:00</v>
+        <v>2026-04-10 15:15:17</v>
       </c>
       <c r="I11" t="str">
         <v/>
@@ -727,16 +723,16 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Bruna Yuculano</v>
+        <v>Adriane Marques</v>
       </c>
       <c r="B12" t="str">
-        <v>sugar1br@gmail.com</v>
+        <v>adrianemarquezcursos@gmail.com</v>
       </c>
       <c r="C12" t="str">
-        <v>Secretaria Municipal de Desenvolvimento Social</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D12" t="str">
-        <v>Psicóloga</v>
+        <v>DCA1</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -745,10 +741,10 @@
         <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G12" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H12" t="str">
-        <v>2026-04-07 20:25:21</v>
+        <v>2026-04-10 15:18:19</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -756,28 +752,28 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Camila Reis</v>
+        <v>Shirley Costa</v>
       </c>
       <c r="B13" t="str">
-        <v>crpereira@pedroleopoldo.mg.gov.br</v>
+        <v>shirley.c14@hotmail.com</v>
       </c>
       <c r="C13" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Governo</v>
       </c>
       <c r="D13" t="str">
-        <v>Coordenadora enfermagem PA central</v>
+        <v>Núcleo de captação de recursos</v>
       </c>
       <c r="E13" t="str">
         <v/>
       </c>
       <c r="F13" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G13" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H13" t="str">
-        <v>2026-04-07 21:44:30</v>
+        <v>2026-04-11 07:24:13</v>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -785,28 +781,28 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Marina de Moura Soares Moura</v>
+        <v>Thais Aparecida</v>
       </c>
       <c r="B14" t="str">
-        <v>marinamourasoares@gmail.com</v>
+        <v>thaisaparecidamtz@hotmail.com</v>
       </c>
       <c r="C14" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D14" t="str">
-        <v>Agente comunitário de saude</v>
+        <v>Analista Administrativo</v>
       </c>
       <c r="E14" t="str">
         <v/>
       </c>
       <c r="F14" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G14" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H14" t="str">
-        <v>2026-04-08 08:34:12</v>
+        <v>2026-04-13 13:44:28</v>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -814,28 +810,28 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Elizabete Dias de Castro</v>
+        <v>Girlene Bastos</v>
       </c>
       <c r="B15" t="str">
-        <v>elizabete.castro@pedroleopoldo.mg.gov.br</v>
+        <v>girlenebarrosobastos@gmail.com</v>
       </c>
       <c r="C15" t="str">
-        <v>Secretaria Municipal de Meio Ambiente</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D15" t="str">
-        <v>Assessora Administrativa</v>
+        <v>Enfermeira</v>
       </c>
       <c r="E15" t="str">
         <v/>
       </c>
       <c r="F15" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G15" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H15" t="str">
-        <v>2026-04-08 09:49:44</v>
+        <v>2026-04-13 14:33:46</v>
       </c>
       <c r="I15" t="str">
         <v/>
@@ -843,28 +839,28 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Sonila Marques</v>
+        <v>Patrícia Pereira de Araújo Fernandes</v>
       </c>
       <c r="B16" t="str">
-        <v>sonila.marques@gmail.com</v>
+        <v>paty2582@gmail.com</v>
       </c>
       <c r="C16" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D16" t="str">
-        <v>Farmacêutica</v>
+        <v>Assistente Administrativo</v>
       </c>
       <c r="E16" t="str">
         <v/>
       </c>
       <c r="F16" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G16" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H16" t="str">
-        <v>2026-04-09 17:04:07</v>
+        <v>2026-04-13 15:14:35</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -872,28 +868,28 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Maria Inês Clemente Bassouto Estevam</v>
+        <v>Andrea Mara da Cruz Rocha</v>
       </c>
       <c r="B17" t="str">
-        <v>maria.estevam@pedroleopoldo.mg.gov.br</v>
+        <v>andrea.rocha@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C17" t="str">
         <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D17" t="str">
-        <v>Gerente de Saúde Ocupacional</v>
+        <v>DCA 11</v>
       </c>
       <c r="E17" t="str">
         <v/>
       </c>
       <c r="F17" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G17" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H17" t="str">
-        <v>2026-04-10 11:04:12</v>
+        <v/>
       </c>
       <c r="I17" t="str">
         <v/>
@@ -901,28 +897,28 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Polyana Parreiras</v>
+        <v>Luciana Nunes Gil</v>
       </c>
       <c r="B18" t="str">
-        <v>PSPARREIRAS@GMAIL.COM</v>
+        <v>luciana.gil@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C18" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Governo</v>
       </c>
       <c r="D18" t="str">
-        <v>Supervisora</v>
+        <v>DCA 6</v>
       </c>
       <c r="E18" t="str">
         <v/>
       </c>
       <c r="F18" t="str">
-        <v>Turma 1 - (Segunda)</v>
+        <v>Turma 2 - (Terça)</v>
       </c>
       <c r="G18" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H18" t="str">
-        <v>2026-04-10 11:04:23</v>
+        <v/>
       </c>
       <c r="I18" t="str">
         <v/>
@@ -930,28 +926,28 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Priscila Malaquias</v>
+        <v>Fabiana Cristina da Silva</v>
       </c>
       <c r="B19" t="str">
-        <v>priscila.malaquiass@gmail.com</v>
+        <v>fabiana.silva@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C19" t="str">
-        <v>Secretaria Municipal de Governo</v>
+        <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D19" t="str">
-        <v>Analista  Administrativo</v>
+        <v>Gerente de Cargos, carreira e desenvolvimento</v>
       </c>
       <c r="E19" t="str">
-        <v/>
+        <v>10013</v>
       </c>
       <c r="F19" t="str">
         <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G19" t="str">
-        <v>Não</v>
+        <v>Sim</v>
       </c>
       <c r="H19" t="str">
-        <v>2026-04-10 11:05:06</v>
+        <v>2026-05-22 12:33:16</v>
       </c>
       <c r="I19" t="str">
         <v/>
@@ -959,16 +955,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Renata Vieira da Silva Dias</v>
+        <v>Ana Paula Silva Diniz</v>
       </c>
       <c r="B20" t="str">
-        <v>red80sam@gmail.com</v>
+        <v>apsd40063@gmail.com</v>
       </c>
       <c r="C20" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Bem Estar</v>
       </c>
       <c r="D20" t="str">
-        <v>Assistente Administrativo</v>
+        <v>DCA 1</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -980,7 +976,7 @@
         <v>Não</v>
       </c>
       <c r="H20" t="str">
-        <v>2026-04-10 11:05:14</v>
+        <v/>
       </c>
       <c r="I20" t="str">
         <v/>
@@ -988,16 +984,16 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Adriana Cristiene Demétrio</v>
+        <v>Elisângel Mesquita de Oliveira</v>
       </c>
       <c r="B21" t="str">
-        <v>adriana.demetrio@pedroleopoldo.mg.gov.br</v>
+        <v>elisangela31mesquita@gmail.com</v>
       </c>
       <c r="C21" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Controladoria Geral do Município</v>
       </c>
       <c r="D21" t="str">
-        <v>Assistente Administrativo</v>
+        <v>Gerente Controle Interno</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -1009,7 +1005,7 @@
         <v>Não</v>
       </c>
       <c r="H21" t="str">
-        <v>2026-04-10 11:12:05</v>
+        <v/>
       </c>
       <c r="I21" t="str">
         <v/>
@@ -1017,28 +1013,28 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Tássia Junqueira</v>
+        <v>Daniela Mara de Oliveira Roberto</v>
       </c>
       <c r="B22" t="str">
-        <v>tassia.junqueira@pedroleopoldo.mg.gov.br</v>
+        <v>danipl22@yahoo.com.br</v>
       </c>
       <c r="C22" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D22" t="str">
-        <v>GERENTE</v>
+        <v>Técnico de Enfermagem</v>
       </c>
       <c r="E22" t="str">
         <v/>
       </c>
       <c r="F22" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G22" t="str">
         <v>Não</v>
       </c>
       <c r="H22" t="str">
-        <v>2026-04-10 14:53:23</v>
+        <v/>
       </c>
       <c r="I22" t="str">
         <v/>
@@ -1046,28 +1042,28 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Ana Beatriz Souza de Jesus</v>
+        <v>Priscilla Gomes Rodrigues</v>
       </c>
       <c r="B23" t="str">
-        <v>ana.jesus@pedroleopoldo.mg.gov.br</v>
+        <v>priscillagomesr@gmail.com</v>
       </c>
       <c r="C23" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D23" t="str">
-        <v>Analista Administrativo</v>
+        <v>Coordenação</v>
       </c>
       <c r="E23" t="str">
         <v/>
       </c>
       <c r="F23" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G23" t="str">
         <v>Não</v>
       </c>
       <c r="H23" t="str">
-        <v>2026-04-10 15:08:22</v>
+        <v/>
       </c>
       <c r="I23" t="str">
         <v/>
@@ -1075,16 +1071,16 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Renata dos Santos Nestor</v>
+        <v>Dirciana Fátima Silva</v>
       </c>
       <c r="B24" t="str">
-        <v>renata.nestor@pedroleopoldo.mg.gov.br</v>
+        <v>dircianafatimademourasilva@gmail.com</v>
       </c>
       <c r="C24" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D24" t="str">
-        <v>DCA 1</v>
+        <v>Auxiliar Administrativo</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -1096,7 +1092,7 @@
         <v>Não</v>
       </c>
       <c r="H24" t="str">
-        <v>2026-04-10 15:12:25</v>
+        <v/>
       </c>
       <c r="I24" t="str">
         <v/>
@@ -1104,28 +1100,28 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Olga Arruda</v>
+        <v>Maria de Fátima Gonçalves Cardoso</v>
       </c>
       <c r="B25" t="str">
-        <v>olga_arruda@hotmail.com</v>
+        <v>mfgcardoso445@gmail.com</v>
       </c>
       <c r="C25" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D25" t="str">
-        <v>Supervisora</v>
+        <v>Agente de saude</v>
       </c>
       <c r="E25" t="str">
         <v/>
       </c>
       <c r="F25" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G25" t="str">
         <v>Não</v>
       </c>
       <c r="H25" t="str">
-        <v>2026-04-10 15:15:17</v>
+        <v/>
       </c>
       <c r="I25" t="str">
         <v/>
@@ -1133,28 +1129,28 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Adriane Marques</v>
+        <v>Lais Macedo Bonfim Rocha</v>
       </c>
       <c r="B26" t="str">
-        <v>adrianemarquezcursos@gmail.com</v>
+        <v>lmbrocha@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C26" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D26" t="str">
-        <v>DCA1</v>
+        <v>Técnica em Radiologia/Supervisora das Técnicas Radiológicas</v>
       </c>
       <c r="E26" t="str">
         <v/>
       </c>
       <c r="F26" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G26" t="str">
         <v>Não</v>
       </c>
       <c r="H26" t="str">
-        <v>2026-04-10 15:18:19</v>
+        <v/>
       </c>
       <c r="I26" t="str">
         <v/>
@@ -1162,16 +1158,16 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Adriele Batista</v>
+        <v>Jeane Fraga dos Santos Pereira</v>
       </c>
       <c r="B27" t="str">
-        <v>adriele.batista@pedroleopoldo.mg.gov.br</v>
+        <v>pereira_jeane2016@yahoo.com.br</v>
       </c>
       <c r="C27" t="str">
-        <v>Secretaria Municipal de Desenvolvimento Social</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D27" t="str">
-        <v>Cadastro Único</v>
+        <v>Técnica de Enfermagem</v>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -1183,7 +1179,7 @@
         <v>Não</v>
       </c>
       <c r="H27" t="str">
-        <v>2026-04-10 16:21:03</v>
+        <v/>
       </c>
       <c r="I27" t="str">
         <v/>
@@ -1191,16 +1187,16 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Fabiana Coutinho</v>
+        <v>Libânia Cássia Alves</v>
       </c>
       <c r="B28" t="str">
-        <v>fafascoutinho@gmail.com</v>
+        <v>libaniacassia@hotmail.com</v>
       </c>
       <c r="C28" t="str">
-        <v>Secretaria Municipal de Desenvolvimento Social</v>
+        <v>Secretaria Municipal de Governo</v>
       </c>
       <c r="D28" t="str">
-        <v>Entrevistador social</v>
+        <v>Coordenadora de projeto</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -1212,7 +1208,7 @@
         <v>Não</v>
       </c>
       <c r="H28" t="str">
-        <v>2026-04-10 16:30:02</v>
+        <v/>
       </c>
       <c r="I28" t="str">
         <v/>
@@ -1220,28 +1216,28 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Luciana Rocha Jorge</v>
+        <v>Bruna Yuculano</v>
       </c>
       <c r="B29" t="str">
-        <v>lucianarjorge@yahoo.com.br</v>
+        <v>sugar1br@gmail.com</v>
       </c>
       <c r="C29" t="str">
-        <v>Secretaria Municipal de Segurança Pública</v>
+        <v>Secretaria Municipal de Desenvolvimento Social</v>
       </c>
       <c r="D29" t="str">
-        <v>Administrativo</v>
+        <v>Psicóloga</v>
       </c>
       <c r="E29" t="str">
         <v/>
       </c>
       <c r="F29" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G29" t="str">
         <v>Não</v>
       </c>
       <c r="H29" t="str">
-        <v>2026-04-10 17:07:48</v>
+        <v/>
       </c>
       <c r="I29" t="str">
         <v/>
@@ -1249,28 +1245,28 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Viviane Catizane do Carmo</v>
+        <v>Camila Reis</v>
       </c>
       <c r="B30" t="str">
-        <v>vcatizanee@gmail.com</v>
+        <v>crpereira@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C30" t="str">
         <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D30" t="str">
-        <v>Enfermeira</v>
+        <v>Coordenadora enfermagem PA central</v>
       </c>
       <c r="E30" t="str">
         <v/>
       </c>
       <c r="F30" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G30" t="str">
         <v>Não</v>
       </c>
       <c r="H30" t="str">
-        <v>2026-04-10 17:18:25</v>
+        <v/>
       </c>
       <c r="I30" t="str">
         <v/>
@@ -1278,28 +1274,28 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Shirley Cosat</v>
+        <v>Marina de Moura Soares</v>
       </c>
       <c r="B31" t="str">
-        <v>shirley.c14@hotmail.com</v>
+        <v>marinamourasoares@gmail.com</v>
       </c>
       <c r="C31" t="str">
-        <v>Secretaria Municipal de Governo</v>
+        <v>Secretaria Municipal de Saúde</v>
       </c>
       <c r="D31" t="str">
-        <v>Núcleo de captação de recursos</v>
+        <v>Agente comunitário de saude</v>
       </c>
       <c r="E31" t="str">
         <v/>
       </c>
       <c r="F31" t="str">
-        <v>Turma 2 - (Terça)</v>
+        <v>Turma 1 - (Segunda)</v>
       </c>
       <c r="G31" t="str">
         <v>Não</v>
       </c>
       <c r="H31" t="str">
-        <v>2026-04-11 07:24:13</v>
+        <v/>
       </c>
       <c r="I31" t="str">
         <v/>
@@ -1307,16 +1303,16 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Marcelle Sena</v>
+        <v>Elizabete Dias de Castro</v>
       </c>
       <c r="B32" t="str">
-        <v>marcelinhasena@hotmail.com</v>
+        <v>elizabete.castro@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C32" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Meio Ambiente</v>
       </c>
       <c r="D32" t="str">
-        <v>Farmacêutica</v>
+        <v>Assessora Administrativa</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -1328,7 +1324,7 @@
         <v>Não</v>
       </c>
       <c r="H32" t="str">
-        <v>2026-04-12 20:17:33</v>
+        <v/>
       </c>
       <c r="I32" t="str">
         <v/>
@@ -1336,16 +1332,16 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Thais Aparecida</v>
+        <v>Renata Vieira da Silva Dias</v>
       </c>
       <c r="B33" t="str">
-        <v>thaisaparecidamtz@hotmail.com</v>
+        <v>red80sam@gmail.com</v>
       </c>
       <c r="C33" t="str">
         <v>Secretaria Municipal de Gestão e Finanças</v>
       </c>
       <c r="D33" t="str">
-        <v>Analista Administrativo</v>
+        <v>Assistente Administrativo</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -1357,7 +1353,7 @@
         <v>Não</v>
       </c>
       <c r="H33" t="str">
-        <v>2026-04-13 13:44:28</v>
+        <v/>
       </c>
       <c r="I33" t="str">
         <v/>
@@ -1365,16 +1361,16 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Girlene Bastos</v>
+        <v>Adriele Batista</v>
       </c>
       <c r="B34" t="str">
-        <v>girlenebarrosobastos@gmail.com</v>
+        <v>adriele.batista@pedroleopoldo.mg.gov.br</v>
       </c>
       <c r="C34" t="str">
-        <v>Secretaria Municipal de Saúde</v>
+        <v>Secretaria Municipal de Desenvolvimento Social</v>
       </c>
       <c r="D34" t="str">
-        <v>Enfermeira</v>
+        <v>Cadastro Único</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -1386,7 +1382,7 @@
         <v>Não</v>
       </c>
       <c r="H34" t="str">
-        <v>2026-04-13 14:33:46</v>
+        <v/>
       </c>
       <c r="I34" t="str">
         <v/>
@@ -1394,16 +1390,16 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Patrícia Barbosa Costa</v>
+        <v>Fabiana Coutinho</v>
       </c>
       <c r="B35" t="str">
-        <v>patpinhati@gmail.com</v>
+        <v>fafascoutinho@gmail.com</v>
       </c>
       <c r="C35" t="str">
-        <v>Secretaria Municipal de Obras</v>
+        <v>Secretaria Municipal de Desenvolvimento Social</v>
       </c>
       <c r="D35" t="str">
-        <v>Assistente Administrativo</v>
+        <v>Entrevistador social</v>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -1415,7 +1411,7 @@
         <v>Não</v>
       </c>
       <c r="H35" t="str">
-        <v>2026-04-13 14:41:35</v>
+        <v/>
       </c>
       <c r="I35" t="str">
         <v/>
@@ -1423,16 +1419,16 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Patrícia Pereira de Araújo Fernandes</v>
+        <v>Luciana Rocha Jorge</v>
       </c>
       <c r="B36" t="str">
-        <v>paty2582@gmail.com</v>
+        <v>lucianarjorge@yahoo.com.br</v>
       </c>
       <c r="C36" t="str">
-        <v>Secretaria Municipal de Gestão e Finanças</v>
+        <v>Secretaria Municipal de Segurança Pública</v>
       </c>
       <c r="D36" t="str">
-        <v>Assistente Administrativo</v>
+        <v>Administrativo</v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -1444,7 +1440,7 @@
         <v>Não</v>
       </c>
       <c r="H36" t="str">
-        <v>2026-04-13 15:14:35</v>
+        <v/>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -1452,37 +1448,124 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v>Viviane Catizane do Carmo</v>
+      </c>
+      <c r="B37" t="str">
+        <v>vcatizanee@gmail.com</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Secretaria Municipal de Saúde</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Enfermeira</v>
+      </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
+      <c r="F37" t="str">
+        <v>Turma 2 - (Terça)</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Não</v>
+      </c>
+      <c r="H37" t="str">
+        <v/>
+      </c>
+      <c r="I37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Marcelle Sena</v>
+      </c>
+      <c r="B38" t="str">
+        <v>marcelinhasena@hotmail.com</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Secretaria Municipal de Saúde</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Farmacêutica</v>
+      </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
+      <c r="F38" t="str">
+        <v>Turma 2 - (Terça)</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Não</v>
+      </c>
+      <c r="H38" t="str">
+        <v/>
+      </c>
+      <c r="I38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Patrícia Barbosa Costa</v>
+      </c>
+      <c r="B39" t="str">
+        <v>patpinhati@gmail.com</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Secretaria Municipal de Obras</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Assistente Administrativo</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
+      </c>
+      <c r="F39" t="str">
+        <v>Turma 2 - (Terça)</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Não</v>
+      </c>
+      <c r="H39" t="str">
+        <v/>
+      </c>
+      <c r="I39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
         <v>Vanessa Macedo Rodrigues</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B40" t="str">
         <v>vanessa.psi1@outlook.com</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C40" t="str">
         <v>Secretaria Municipal de Desenvolvimento Social</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D40" t="str">
         <v>Psicóloga</v>
       </c>
-      <c r="E37" t="str">
-        <v/>
-      </c>
-      <c r="F37" t="str">
-        <v>Turma 2 - (Terça)</v>
-      </c>
-      <c r="G37" t="str">
-        <v>Não</v>
-      </c>
-      <c r="H37" t="str">
-        <v>2026-04-13 17:45:01</v>
-      </c>
-      <c r="I37" t="str">
+      <c r="E40" t="str">
+        <v/>
+      </c>
+      <c r="F40" t="str">
+        <v>Turma 2 - (Terça)</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Não</v>
+      </c>
+      <c r="H40" t="str">
+        <v/>
+      </c>
+      <c r="I40" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I37"/>
+  <autoFilter ref="A1:I40"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I40"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>